<commit_message>
mejora del chatbot y boton de recargar
</commit_message>
<xml_diff>
--- a/data/pedidos_2026-08-11.xlsx
+++ b/data/pedidos_2026-08-11.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedidos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pedidos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,6 +498,1725 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1. Milagro Elizabeth Segovia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>77375251</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>San Miguel</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SAN MIGUEL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Colonia panorama calle principal #17</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>wood negro
+wood cafe</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2. Marina</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>73118941</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cabañas</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ILOBASCO</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Universidad Católica de El Salvador </t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Rose Gold Mini</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3. Jose Edgardo Sanchez Tel</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>76839773</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>San Miguel</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SAN MIGUEL</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12 calle poniente 109 barrio san francisco San Miguel centro. </t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>- MRW200H Azul fondo Blanco
+ -MRW200H Full Negro</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4. Melanie Paola Palacios Cruz</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>64419003</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>San Salvador</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SANTO TOMAS</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Carretera Antigua a Zacatecoluca. Km 9. Colonia Moran. Casa #3. Santo Tomás, San Salvador.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rose Gold RETRO
+</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5. María del Carmen Girón de Polio</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>78783041</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>San Miguel</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CHINAMECA</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FPFG+M5X Conacastal, Chinameca, Departamento de San Miguel.
+</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Llantería Cáceres.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>RETRO Black</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6. Jose Enrique Guerra Guerra Num.</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>75148839</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Chalatenango</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AGUA CALIENTE</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>el centro agua caliente chalatenango por farmacias popular en SG MOTOS AG.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Rose Gold Mini</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>7. Sonia Delgado</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>71678946</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Santa Ana</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>EL CONGO</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cantón la presa.
+</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Rose Gold DIAMOND</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>8. Ana Lissette Quinteros</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>60177851</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Santa Ana</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SANTA ANA</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Final 6av norte, senda 1 poniente, block D, casa 11, Residencial Río Zarco, contiguo a residencial alameda</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Sin referencia</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2 relojes - Casio LTP E 117 negro</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>9. juan carlos Reyes</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>79311237</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Morazán</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CORINTO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>parque central de corinto</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>RETRO Black</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>10. Rebecca Sarai Martinez Cuellar</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>73923176</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>La Paz</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SAN PEDRO MASAHUAT</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Colonia villas de san pedro, poligono G casa 2</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Cerca del aeropuerto Monseñor Romero, carretera a playa las hojas</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Old Money Rose Gold</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>11. María dora Toloza</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>77389099</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>San Vicente</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TECOLUCA</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>col san romero, casa 7</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> a la par de tieda matoya me conocen cómo niña Doris.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Rose Gold DIAMOND</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>12. Rebeca Marisela Escobar Martinez</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>60376347</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>San Salvador</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SAN MARCOS</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Carretera a comalapa kilómetro 11 ½, Colonia san Antonio Guadalupe pasaje Belén casa número #7 san marcos, san salvador</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Punto de referencia: enfrente de fábrica FAMENSAL</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Old Money Rose Gold</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>13. Sandy Tatiana Meléndez Ayala</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>79537408</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>La Libertad</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>QUEZALTEPEQUE</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Gasolinera uno quezaltepeque</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>RPFG+F6W, Quezaltepeque</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Retro Black</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>14. Genesis Paola Franco Serpas</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>61495494</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Usulután</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>USULUTAN</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Calle Federico Penado #12, Barrio La Merced, Usulután Usulutan CP, 3401, Tartaleta Café y Bistro</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>banco promerica.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Rose Gold DIAMOND</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Si se entrega miercoles, que se entregue antes de las 12(por la mañana) y se entrega jueves que sea por la tarde</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>15. maría ines flores arteaga</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>69949348</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Cuscatlán</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>SUCHITOTO</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carretera hacia suchitoto cantón Bermuda comunidad las américa colonia buena vista
+La colonia esta ubicada después de el desvío de la Bermuda y antes de el desvío de ciudadela  
+</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Centro de formación Cordes Region 2</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Casio rosegold diamond</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>16. Mery de Henriquez</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>70164612</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Sonsonate</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NAHULINGO</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Colonia entre ríos block 2 lote 14 nahuilingo</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>rose gold retro</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>17. Jesus Andersson Franco Hernández</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>75049461</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>La Paz</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SAN LUIS TALPA</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Kilómetro 42½ sobre la Autopista de Comalapa, el lugar se llama Vaquerano Rent a Car</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Referencia: Frente a el control policial de entrada al Aeropuerto</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Casio f105</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>27.00</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>18. Efrain lopez</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>78606698</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Usulután</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>SANTA ELENA</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>frente a la iglesia, parque de santa elena</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Casio World</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>19. Roberto Marroquin</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>76102396</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Santa Ana</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CHALCHUAPA</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 calle poniente casa numero 2 </t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>frente caja de credito barrio san sebastian distrito</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Aviador negro Aviador dorado 2x1</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20. Gloria Guzman</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>79383931</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Santa Ana</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>SANTA ANA</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>unidad de salud san rafael la del ministerio</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>queda en la bajada para unicaes santa ana</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Promocion Wood negro y aviador negro</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>21. Angelly Rossibel Reyes Maltez</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>77877516</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>San Miguel</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>SAN MIGUEL</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Colonia 14 de Julio, Calle concepcion casa #3</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>seiko 5 fondo negro</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Cambio!!! clienta entrega reloj</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>22. Esperanza Gonzaleź</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>70498368</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Santa Ana</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>CHALCHUAPA</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Santa ana municipio de chalchuapa, 2a Calle Ote. 9-A, Chalchuapa 2205</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>referencia: Farmacias Económicas - Chalchuapa</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Aviador negro 
+wood cafe</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>23. Heidy Saravia</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>70482669</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>La Libertad</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>SANTA TECLA</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>centro comercial la joya</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> en banco davivienda</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Casio Old Money Rose gold</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega, Entrega entre las 9am y 5 pm</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>24. Josue Morales</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>74313159</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>La Libertad</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>COLON</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Urbanización Nuevo Lourdes</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Frente a casa comunal</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Aviador Negro
+Aviador dorado</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>25. Hizer Alvarez Salgado</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>74968695</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>San Miguel</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>SAN MIGUEL</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>4ta calle poniente 705</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Universidad de Oriente</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Casio MRW-200H full negro</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar a la entrega</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>